<commit_message>
Golf 2026-04-04: run pipeline scripts + postplanner exports
Re-ran verify-facts (52 claims, 93 HIGH), compile-content-data,
generate-review-dashboard (31 items), and postplanner exports (11 posts
standard + TOBI). WordPress publish blocked by egress proxy.

https://claude.ai/code/session_01Wrhtkf9PRGJD5yX5hYKVTc
</commit_message>
<xml_diff>
--- a/Golf/postplanner-imports/gfr-postplanner-2026-04-04.xlsx
+++ b/Golf/postplanner-imports/gfr-postplanner-2026-04-04.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/04/2026  17:37</t>
+          <t>04/04/2026  18:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -494,7 +494,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/04/2026  18:00</t>
+          <t>04/04/2026  18:45</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -512,7 +512,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/04/2026  18:23</t>
+          <t>04/04/2026  19:04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/04/2026  18:46</t>
+          <t>04/04/2026  19:23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -544,7 +544,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/04/2026  19:09</t>
+          <t>04/04/2026  19:42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/04/2026  19:32</t>
+          <t>04/04/2026  20:01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -578,7 +578,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/04/2026  19:55</t>
+          <t>04/04/2026  20:20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -594,7 +594,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/04/2026  20:18</t>
+          <t>04/04/2026  20:39</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -610,7 +610,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04/04/2026  20:41</t>
+          <t>04/04/2026  20:58</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -625,7 +625,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04/04/2026  21:04</t>
+          <t>04/04/2026  21:17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04/04/2026  21:27</t>
+          <t>04/04/2026  21:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">

</xml_diff>